<commit_message>
redid all analyses with the new parental-daughter copy dataset
</commit_message>
<xml_diff>
--- a/data/tissueCorr.xlsx
+++ b/data/tissueCorr.xlsx
@@ -1422,55 +1422,55 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>139</v>
+        <v>48</v>
       </c>
       <c r="C18" t="n">
-        <v>0.8022792966390503</v>
+        <v>0.591537068118644</v>
       </c>
       <c r="D18" t="n">
-        <v>1.69876772689362e-32</v>
+        <v>9.528734198891293e-06</v>
       </c>
       <c r="E18" t="n">
-        <v>0.8034183022761963</v>
+        <v>0.6139565238526075</v>
       </c>
       <c r="F18" t="n">
-        <v>1.192491651919879e-32</v>
+        <v>3.469934030167387e-06</v>
       </c>
       <c r="G18" t="n">
-        <v>0.8091556681373349</v>
+        <v>0.7292022975165409</v>
       </c>
       <c r="H18" t="n">
-        <v>1.935325663505403e-33</v>
+        <v>4.159059753724258e-09</v>
       </c>
       <c r="I18" t="n">
-        <v>0.748489095619712</v>
+        <v>0.6008196999116411</v>
       </c>
       <c r="J18" t="n">
-        <v>3.286510847740087e-26</v>
+        <v>6.330233632434536e-06</v>
       </c>
       <c r="K18" t="n">
-        <v>0.7841878960600329</v>
+        <v>0.5149417847273063</v>
       </c>
       <c r="L18" t="n">
-        <v>3.50190645992558e-30</v>
+        <v>0.0001805140496860693</v>
       </c>
       <c r="M18" t="n">
-        <v>0.7824115802366799</v>
+        <v>0.6152551719441804</v>
       </c>
       <c r="N18" t="n">
-        <v>5.747682013990053e-30</v>
+        <v>3.264874800332008e-06</v>
       </c>
       <c r="O18" t="n">
-        <v>0.764948216575413</v>
+        <v>0.65145375652732</v>
       </c>
       <c r="P18" t="n">
-        <v>5.92666289152679e-28</v>
+        <v>5.317386020619207e-07</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.7876548754347066</v>
+        <v>0.5702497420013828</v>
       </c>
       <c r="R18" t="n">
-        <v>1.31337551574387e-30</v>
+        <v>2.324046513866802e-05</v>
       </c>
     </row>
     <row r="19">
@@ -1480,55 +1480,55 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>170</v>
+        <v>51</v>
       </c>
       <c r="C19" t="n">
-        <v>0.3405755277271076</v>
+        <v>0.3322316870125145</v>
       </c>
       <c r="D19" t="n">
-        <v>5.509107450013463e-06</v>
+        <v>0.01722444738896729</v>
       </c>
       <c r="E19" t="n">
-        <v>0.3988562093202984</v>
+        <v>0.3581745538233855</v>
       </c>
       <c r="F19" t="n">
-        <v>7.150668523206573e-08</v>
+        <v>0.009859759389413121</v>
       </c>
       <c r="G19" t="n">
-        <v>0.4612899987067662</v>
+        <v>0.2581156783399217</v>
       </c>
       <c r="H19" t="n">
-        <v>2.439813266704579e-10</v>
+        <v>0.06743826229117293</v>
       </c>
       <c r="I19" t="n">
-        <v>0.4226895982747765</v>
+        <v>0.3454068602096585</v>
       </c>
       <c r="J19" t="n">
-        <v>9.358612480078351e-09</v>
+        <v>0.01304734734550875</v>
       </c>
       <c r="K19" t="n">
-        <v>0.4498435330391691</v>
+        <v>0.2723321882502419</v>
       </c>
       <c r="L19" t="n">
-        <v>7.548244186416661e-10</v>
+        <v>0.05319412413572143</v>
       </c>
       <c r="M19" t="n">
-        <v>0.4781389561523639</v>
+        <v>0.4416273208555694</v>
       </c>
       <c r="N19" t="n">
-        <v>4.280981159473087e-11</v>
+        <v>0.001177774666596081</v>
       </c>
       <c r="O19" t="n">
-        <v>0.4214430376473137</v>
+        <v>0.4128404320704501</v>
       </c>
       <c r="P19" t="n">
-        <v>1.04502541008777e-08</v>
+        <v>0.002606233435317057</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.4142563586848992</v>
+        <v>0.2619247540649445</v>
       </c>
       <c r="R19" t="n">
-        <v>1.957053365926218e-08</v>
+        <v>0.06335309191059732</v>
       </c>
     </row>
     <row r="20">
@@ -1538,55 +1538,55 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>364</v>
+        <v>100</v>
       </c>
       <c r="C20" t="n">
-        <v>0.7358848682603839</v>
+        <v>0.5810312993105302</v>
       </c>
       <c r="D20" t="n">
-        <v>2.833622570198045e-63</v>
+        <v>2.33266968345512e-10</v>
       </c>
       <c r="E20" t="n">
-        <v>0.7369704319381802</v>
+        <v>0.4657038108836767</v>
       </c>
       <c r="F20" t="n">
-        <v>1.503468610002566e-63</v>
+        <v>1.047622443102353e-06</v>
       </c>
       <c r="G20" t="n">
-        <v>0.735499738743905</v>
+        <v>0.52366118494444</v>
       </c>
       <c r="H20" t="n">
-        <v>3.545404382690163e-63</v>
+        <v>2.26335213873931e-08</v>
       </c>
       <c r="I20" t="n">
-        <v>0.7278063054173988</v>
+        <v>0.4923883091824421</v>
       </c>
       <c r="J20" t="n">
-        <v>2.875748409302417e-61</v>
+        <v>1.956628878923379e-07</v>
       </c>
       <c r="K20" t="n">
-        <v>0.7272387513065205</v>
+        <v>0.3695405074477543</v>
       </c>
       <c r="L20" t="n">
-        <v>3.953622223622513e-61</v>
+        <v>0.0001544540393053403</v>
       </c>
       <c r="M20" t="n">
-        <v>0.7256454313861814</v>
+        <v>0.5363761270613293</v>
       </c>
       <c r="N20" t="n">
-        <v>9.621353293057456e-61</v>
+        <v>8.832533789436949e-09</v>
       </c>
       <c r="O20" t="n">
-        <v>0.7280474994813434</v>
+        <v>0.4713955113560506</v>
       </c>
       <c r="P20" t="n">
-        <v>2.511280261517744e-61</v>
+        <v>7.411557303141777e-07</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.6830590382567332</v>
+        <v>0.4443572225667455</v>
       </c>
       <c r="R20" t="n">
-        <v>2.440853132328556e-51</v>
+        <v>3.63382145539626e-06</v>
       </c>
     </row>
     <row r="21">
@@ -1596,55 +1596,55 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>478</v>
+        <v>80</v>
       </c>
       <c r="C21" t="n">
-        <v>0.3959342744279958</v>
+        <v>0.2931258883022751</v>
       </c>
       <c r="D21" t="n">
-        <v>2.169848346771814e-19</v>
+        <v>0.008320778311627626</v>
       </c>
       <c r="E21" t="n">
-        <v>0.4490237976037242</v>
+        <v>0.3256779159393632</v>
       </c>
       <c r="F21" t="n">
-        <v>4.292420391845935e-25</v>
+        <v>0.003199129080836441</v>
       </c>
       <c r="G21" t="n">
-        <v>0.4165319243497081</v>
+        <v>0.1999789017312331</v>
       </c>
       <c r="H21" t="n">
-        <v>1.749762863743589e-21</v>
+        <v>0.07531733025947505</v>
       </c>
       <c r="I21" t="n">
-        <v>0.415532041214385</v>
+        <v>0.2635389069078931</v>
       </c>
       <c r="J21" t="n">
-        <v>2.228395059174749e-21</v>
+        <v>0.0181774067131736</v>
       </c>
       <c r="K21" t="n">
-        <v>0.444749639269974</v>
+        <v>0.2115616872225251</v>
       </c>
       <c r="L21" t="n">
-        <v>1.349480322957733e-24</v>
+        <v>0.05958284216726146</v>
       </c>
       <c r="M21" t="n">
-        <v>0.415807979209362</v>
+        <v>0.3238895040741049</v>
       </c>
       <c r="N21" t="n">
-        <v>2.084716036837048e-21</v>
+        <v>0.003380865015432705</v>
       </c>
       <c r="O21" t="n">
-        <v>0.3388582238253975</v>
+        <v>0.1912881082104087</v>
       </c>
       <c r="P21" t="n">
-        <v>2.624791676078184e-14</v>
+        <v>0.08917986615569978</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.386051994092302</v>
+        <v>0.3221780666169964</v>
       </c>
       <c r="R21" t="n">
-        <v>1.950141865163154e-18</v>
+        <v>0.003563352070204926</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tau and number of tissue correlations with retrogenes and enriched GO terms removed as well
</commit_message>
<xml_diff>
--- a/data/tissueCorr.xlsx
+++ b/data/tissueCorr.xlsx
@@ -413,10 +413,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
       <c r="C1" t="inlineStr">
         <is>
           <t>Brain</t>
@@ -455,6 +460,11 @@
       <c r="Q1" t="inlineStr">
         <is>
           <t>Stomach</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -544,6 +554,26 @@
           <t>P</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Tau</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Tau PValue</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Num Tissues</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Num Tissues PValue</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -552,7 +582,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16118</v>
+        <v>15891</v>
       </c>
       <c r="C3" t="n">
         <v>0.8239536052601645</v>
@@ -602,6 +632,18 @@
       <c r="R3" t="n">
         <v>0</v>
       </c>
+      <c r="S3" t="n">
+        <v>0.6947566471394999</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.7768062651179639</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -610,7 +652,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1887</v>
+        <v>1210</v>
       </c>
       <c r="C4" t="n">
         <v>0.4836366105085619</v>
@@ -660,6 +702,18 @@
       <c r="R4" t="n">
         <v>4.091754947066972e-118</v>
       </c>
+      <c r="S4" t="n">
+        <v>0.4795044550892388</v>
+      </c>
+      <c r="T4" t="n">
+        <v>1.396174251195149e-70</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.4453733055078301</v>
+      </c>
+      <c r="V4" t="n">
+        <v>6.655207393402821e-98</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -668,7 +722,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>480</v>
+        <v>419</v>
       </c>
       <c r="C5" t="n">
         <v>0.5232568651948065</v>
@@ -718,6 +772,18 @@
       <c r="R5" t="n">
         <v>5.997891724564006e-39</v>
       </c>
+      <c r="S5" t="n">
+        <v>0.5671658235283655</v>
+      </c>
+      <c r="T5" t="n">
+        <v>4.900634509550861e-37</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.467637136667817</v>
+      </c>
+      <c r="V5" t="n">
+        <v>2.910889828002275e-28</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -726,7 +792,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>221</v>
+        <v>185</v>
       </c>
       <c r="C6" t="n">
         <v>0.3342825711899206</v>
@@ -776,6 +842,18 @@
       <c r="R6" t="n">
         <v>5.982434394029979e-09</v>
       </c>
+      <c r="S6" t="n">
+        <v>0.4111990685095912</v>
+      </c>
+      <c r="T6" t="n">
+        <v>6.090475886142049e-09</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.3492232584821083</v>
+      </c>
+      <c r="V6" t="n">
+        <v>5.339805938636754e-08</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -784,7 +862,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C7" t="n">
         <v>0.7676330385274209</v>
@@ -834,6 +912,18 @@
       <c r="R7" t="n">
         <v>4.95209166998049e-08</v>
       </c>
+      <c r="S7" t="n">
+        <v>0.35869376660426</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.03169217508223911</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0.5165576146523634</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.0001042440114676383</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -842,7 +932,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C8" t="n">
         <v>0.5137598459867665</v>
@@ -892,6 +982,18 @@
       <c r="R8" t="n">
         <v>2.209627631562022e-09</v>
       </c>
+      <c r="S8" t="n">
+        <v>0.729610473438415</v>
+      </c>
+      <c r="T8" t="n">
+        <v>5.430229907274177e-12</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.4575093846627829</v>
+      </c>
+      <c r="V8" t="n">
+        <v>7.740575889689321e-05</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -900,7 +1002,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C9" t="n">
         <v>0.8103248578784161</v>
@@ -950,6 +1052,18 @@
       <c r="R9" t="n">
         <v>4.184823363044267e-07</v>
       </c>
+      <c r="S9" t="n">
+        <v>0.8016164506652007</v>
+      </c>
+      <c r="T9" t="n">
+        <v>1.460861960690243e-06</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.7615895421772363</v>
+      </c>
+      <c r="V9" t="n">
+        <v>2.511428752441402e-06</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -958,7 +1072,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="C10" t="n">
         <v>0.7295687312515601</v>
@@ -1008,6 +1122,18 @@
       <c r="R10" t="n">
         <v>3.929877245842215e-20</v>
       </c>
+      <c r="S10" t="n">
+        <v>0.7633897538012618</v>
+      </c>
+      <c r="T10" t="n">
+        <v>7.636974790046126e-22</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.7469300447196769</v>
+      </c>
+      <c r="V10" t="n">
+        <v>4.089299234692123e-22</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1016,7 +1142,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1405</v>
+        <v>789</v>
       </c>
       <c r="C11" t="n">
         <v>0.542692406410337</v>
@@ -1066,6 +1192,18 @@
       <c r="R11" t="n">
         <v>1.493887510955844e-112</v>
       </c>
+      <c r="S11" t="n">
+        <v>0.4281890409795512</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1.60983453221445e-36</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.5182040388601888</v>
+      </c>
+      <c r="V11" t="n">
+        <v>7.578889427263108e-104</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1074,7 +1212,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>567</v>
+        <v>259</v>
       </c>
       <c r="C12" t="n">
         <v>0.3375604659237577</v>
@@ -1124,6 +1262,18 @@
       <c r="R12" t="n">
         <v>2.144593877891096e-17</v>
       </c>
+      <c r="S12" t="n">
+        <v>0.3870541917637939</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1.102744017468685e-10</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.2846284022689176</v>
+      </c>
+      <c r="V12" t="n">
+        <v>3.03911737241696e-13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1132,7 +1282,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>143</v>
+        <v>57</v>
       </c>
       <c r="C13" t="n">
         <v>0.617529506248037</v>
@@ -1182,6 +1332,18 @@
       <c r="R13" t="n">
         <v>4.922430660559533e-12</v>
       </c>
+      <c r="S13" t="n">
+        <v>0.3289076818865542</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0.01248554433479151</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.57892890137978</v>
+      </c>
+      <c r="V13" t="n">
+        <v>1.285787024537455e-14</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1190,7 +1352,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>198</v>
+        <v>103</v>
       </c>
       <c r="C14" t="n">
         <v>0.6132039338427117</v>
@@ -1240,6 +1402,18 @@
       <c r="R14" t="n">
         <v>2.025850663314799e-19</v>
       </c>
+      <c r="S14" t="n">
+        <v>0.39905161059371</v>
+      </c>
+      <c r="T14" t="n">
+        <v>2.975578897563617e-05</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.5365886931399939</v>
+      </c>
+      <c r="V14" t="n">
+        <v>1.562097375815211e-16</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1248,7 +1422,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>122</v>
+        <v>52</v>
       </c>
       <c r="C15" t="n">
         <v>0.6745213535176455</v>
@@ -1298,6 +1472,18 @@
       <c r="R15" t="n">
         <v>3.405555502739186e-21</v>
       </c>
+      <c r="S15" t="n">
+        <v>0.4168448663564142</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0.002111442761072418</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0.7708548107801908</v>
+      </c>
+      <c r="V15" t="n">
+        <v>3.031760752857564e-26</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1306,7 +1492,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>375</v>
+        <v>318</v>
       </c>
       <c r="C16" t="n">
         <v>0.6758942503121481</v>
@@ -1356,6 +1542,18 @@
       <c r="R16" t="n">
         <v>9.099786985374136e-49</v>
       </c>
+      <c r="S16" t="n">
+        <v>0.4849830219427531</v>
+      </c>
+      <c r="T16" t="n">
+        <v>3.643280656351324e-20</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0.6792385386919162</v>
+      </c>
+      <c r="V16" t="n">
+        <v>4.416510571271564e-54</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1364,7 +1562,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4008</v>
+        <v>1189</v>
       </c>
       <c r="C17" t="n">
         <v>0.4131103463464055</v>
@@ -1414,6 +1612,18 @@
       <c r="R17" t="n">
         <v>9.307728654583262e-182</v>
       </c>
+      <c r="S17" t="n">
+        <v>0.1592890019337498</v>
+      </c>
+      <c r="T17" t="n">
+        <v>3.34971176414662e-08</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0.5437370598105713</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1472,6 +1682,18 @@
       <c r="R18" t="n">
         <v>2.324046513866802e-05</v>
       </c>
+      <c r="S18" t="n">
+        <v>0.7857123542212767</v>
+      </c>
+      <c r="T18" t="n">
+        <v>3.733283279428872e-11</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0.6180374548869156</v>
+      </c>
+      <c r="V18" t="n">
+        <v>2.862779512605718e-06</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1530,6 +1752,18 @@
       <c r="R19" t="n">
         <v>0.06335309191059732</v>
       </c>
+      <c r="S19" t="n">
+        <v>0.5985422325300412</v>
+      </c>
+      <c r="T19" t="n">
+        <v>3.497887250433168e-06</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0.3526415748507207</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.0111473757019604</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1588,6 +1822,18 @@
       <c r="R20" t="n">
         <v>3.63382145539626e-06</v>
       </c>
+      <c r="S20" t="n">
+        <v>0.6799072237818248</v>
+      </c>
+      <c r="T20" t="n">
+        <v>7.334173742261159e-15</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0.6235909814419237</v>
+      </c>
+      <c r="V20" t="n">
+        <v>4.211474154410818e-12</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1646,9 +1892,21 @@
       <c r="R21" t="n">
         <v>0.003563352070204926</v>
       </c>
+      <c r="S21" t="n">
+        <v>0.430358388654927</v>
+      </c>
+      <c r="T21" t="n">
+        <v>6.763641215353774e-05</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0.3060262282821574</v>
+      </c>
+      <c r="V21" t="n">
+        <v>0.00576831712211481</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="Q1:R1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="G1:H1"/>
@@ -1657,6 +1915,7 @@
     <mergeCell ref="O1:P1"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="I1:J1"/>
+    <mergeCell ref="S1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>